<commit_message>
Add professional Resume template and technical bullet points for Advance Excel & MIS Specialist
</commit_message>
<xml_diff>
--- a/Excel Formulas .xlsx
+++ b/Excel Formulas .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lucky\Desktop\Advance Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7535FDD5-492F-48A1-BEFA-95DC517B3651}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{00F5FB19-61BE-4111-91E0-3E33A674F916}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-105" yWindow="-105" windowWidth="23250" windowHeight="12720" tabRatio="913" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3559,14 +3559,14 @@
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="41">
         <f ca="1">TODAY()</f>
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="B3">
         <v>7</v>
       </c>
       <c r="C3" s="41">
         <f ca="1">A3+B3</f>
-        <v>46252</v>
+        <v>46259</v>
       </c>
       <c r="D3" t="s">
         <v>221</v>
@@ -3575,20 +3575,20 @@
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="41">
         <f ca="1">TODAY()</f>
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="B4">
         <v>5</v>
       </c>
       <c r="C4" s="41">
         <f ca="1">A4-B4</f>
-        <v>46240</v>
+        <v>46247</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="50">
         <f ca="1">NOW()</f>
-        <v>46245.642577662038</v>
+        <v>46252.847921875</v>
       </c>
       <c r="C6" t="s">
         <v>222</v>
@@ -3615,7 +3615,7 @@
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10">
         <f ca="1">DAY(A6)</f>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
         <v>225</v>
@@ -3624,7 +3624,7 @@
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="41">
         <f ca="1">DATE(A8,A9,A10)</f>
-        <v>46245</v>
+        <v>46252</v>
       </c>
       <c r="C12" t="s">
         <v>226</v>
@@ -3659,7 +3659,7 @@
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="str">
         <f ca="1">TEXT(A12,"dd")</f>
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="B16" t="str">
         <f ca="1">TEXT(A6,"mm")</f>
@@ -5757,11 +5757,11 @@
       </c>
       <c r="F24" s="38">
         <f t="shared" ref="D24:G35" ca="1" si="0">RANDBETWEEN(5000,50000)</f>
-        <v>15093</v>
+        <v>13072</v>
       </c>
       <c r="G24" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>22169</v>
+        <v>20139</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
@@ -5779,11 +5779,11 @@
       </c>
       <c r="F25" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>14811</v>
+        <v>42833</v>
       </c>
       <c r="G25" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>18109</v>
+        <v>26623</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
@@ -5796,11 +5796,11 @@
       </c>
       <c r="F26" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>19734</v>
+        <v>47537</v>
       </c>
       <c r="G26" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>12095</v>
+        <v>11022</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
@@ -5813,11 +5813,11 @@
       </c>
       <c r="F27" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>44869</v>
+        <v>35730</v>
       </c>
       <c r="G27" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>30059</v>
+        <v>33489</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
@@ -5828,11 +5828,11 @@
       </c>
       <c r="F28" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>7598</v>
+        <v>36939</v>
       </c>
       <c r="G28" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>6790</v>
+        <v>27128</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.25">
@@ -5840,41 +5840,41 @@
       <c r="C29" s="35"/>
       <c r="F29" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>10065</v>
+        <v>37837</v>
       </c>
       <c r="G29" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>8684</v>
+        <v>45525</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="33"/>
       <c r="C30" s="38">
         <f ca="1">RANDBETWEEN(5000,50000)</f>
-        <v>33407</v>
+        <v>44443</v>
       </c>
       <c r="D30" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>16353</v>
+        <v>35197</v>
       </c>
       <c r="E30" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>11281</v>
+        <v>7927</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="21" x14ac:dyDescent="0.35">
       <c r="A31" s="33"/>
       <c r="C31" s="38">
         <f t="shared" ref="C31:C35" ca="1" si="1">RANDBETWEEN(5000,50000)</f>
-        <v>37868</v>
+        <v>40796</v>
       </c>
       <c r="D31" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>38868</v>
+        <v>28881</v>
       </c>
       <c r="E31" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>14511</v>
+        <v>16302</v>
       </c>
       <c r="G31" s="39" t="s">
         <v>151</v>
@@ -5884,60 +5884,60 @@
       <c r="A32" s="33"/>
       <c r="C32" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>12253</v>
+        <v>8089</v>
       </c>
       <c r="D32" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>19642</v>
+        <v>6895</v>
       </c>
       <c r="E32" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>5335</v>
+        <v>6028</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="33"/>
       <c r="C33" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>11898</v>
+        <v>14143</v>
       </c>
       <c r="D33" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>48982</v>
+        <v>26770</v>
       </c>
       <c r="E33" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>9847</v>
+        <v>38279</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" s="34"/>
       <c r="C34" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>15201</v>
+        <v>43445</v>
       </c>
       <c r="D34" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>48204</v>
+        <v>11845</v>
       </c>
       <c r="E34" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>26260</v>
+        <v>12726</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" s="34"/>
       <c r="C35" s="38">
         <f t="shared" ca="1" si="1"/>
-        <v>26953</v>
+        <v>41977</v>
       </c>
       <c r="D35" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>20955</v>
+        <v>33719</v>
       </c>
       <c r="E35" s="38">
         <f t="shared" ca="1" si="0"/>
-        <v>25756</v>
+        <v>8915</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">

</xml_diff>